<commit_message>
Publish Deal Decoded #2: Sun Pharma / Organon (posted 29-Oct-2026)
- deal card live; note, model and key numbers as of the 28-Oct-2026 close
- adds the ACCC review (Phase 1 ends 3-Dec-2026, ganirelix remedy) to the note
- bump data.js cache version

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B7AfZPuoisxdHY8WGcdvpp
</commit_message>
<xml_diff>
--- a/assets/files/deal-sun-pharma-organon-model.xlsx
+++ b/assets/files/deal-sun-pharma-organon-model.xlsx
@@ -31,12 +31,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="524" uniqueCount="494">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="497">
   <si>
     <t xml:space="preserve">DEAL DECODED #2 · SUN PHARMA / ORGANON</t>
   </si>
   <si>
-    <t xml:space="preserve">Outside-in analysis from public filings. Debjit Mukherjee, IB Independent. Market data to 23-Oct-2026. Live deal — not investment advice.</t>
+    <t xml:space="preserve">Outside-in analysis from public filings. Debjit Mukherjee, IB Independent. Market data to 28-Oct-2026. Live deal — not investment advice.</t>
   </si>
   <si>
     <t xml:space="preserve">HEADLINE OUTPUTS</t>
@@ -201,7 +201,7 @@
     <t xml:space="preserve">Approvals outstanding</t>
   </si>
   <si>
-    <t xml:space="preserve">Non-US antitrust, foreign direct investment and EU Foreign Subsidies Regulation clearances. HSR filed 21-May-2026, waiting period scheduled to expire 22-Jun-2026 (no later filing mentions HSR). Sun also has Indian overseas-investment filings to make</t>
+    <t xml:space="preserve">Non-US antitrust, foreign direct investment and EU Foreign Subsidies Regulation clearances. HSR filed 21-May-2026, waiting period scheduled to expire 22-Jun-2026 (no later filing mentions HSR). Sun also has Indian overseas-investment filings to make. Australia (ACCC MN-35035): notified 22-Oct-2026, Phase 1 ends 3-Dec-2026; Sun has offered to license its generic ganirelix in Australia to Ferring</t>
   </si>
   <si>
     <t xml:space="preserve">Organon advisers</t>
@@ -540,10 +540,10 @@
     <t xml:space="preserve">Sun Pharma (acquirer) — standalone</t>
   </si>
   <si>
-    <t xml:space="preserve">Source: desk Sun Pharma model (COVERAGE/SUN PHARMA, published 07-Sep-2026, built from company filings); prices NSE close 23-Oct-2026; Sun investor call 27-Apr-2026.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Share price, 23-Oct-2026 (Rs)</t>
+    <t xml:space="preserve">Source: desk Sun Pharma model (COVERAGE/SUN PHARMA, published 07-Sep-2026, built from company filings); prices NSE close 28-Oct-2026; Sun investor call 27-Apr-2026.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Share price, 28-Oct-2026 (Rs)</t>
   </si>
   <si>
     <t xml:space="preserve">Shares outstanding (crore)</t>
@@ -585,7 +585,7 @@
     <t xml:space="preserve">Trailing P/E (x)</t>
   </si>
   <si>
-    <t xml:space="preserve">USD/INR, 23-Oct-2026</t>
+    <t xml:space="preserve">USD/INR, 28-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">USD/INR, 27-Apr-2026 (announcement)</t>
@@ -966,7 +966,7 @@
     <t xml:space="preserve">Sources &amp; uses, pro forma leverage</t>
   </si>
   <si>
-    <t xml:space="preserve">US$ millions; rupee figures converted at the 23-Oct-2026 rate.</t>
+    <t xml:space="preserve">US$ millions; rupee figures converted at the 28-Oct-2026 rate.</t>
   </si>
   <si>
     <t xml:space="preserve">Sources</t>
@@ -1038,10 +1038,10 @@
     <t xml:space="preserve">Live deal — merger-arbitrage spread and the odds the market is pricing</t>
   </si>
   <si>
-    <t xml:space="preserve">Prices: NYSE close 23-Oct-2026. Expected close and break price are desk assumptions (blue). Refresh on the day of posting.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">OGN close, 23-Oct-2026 ($)</t>
+    <t xml:space="preserve">Prices: NYSE close 28-Oct-2026. Expected close and break price are desk assumptions (blue). Refresh on the day of posting.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">OGN close, 28-Oct-2026 ($)</t>
   </si>
   <si>
     <t xml:space="preserve">Dividends expected before close ($, $0.02 quarterly)</t>
@@ -1065,7 +1065,7 @@
     <t xml:space="preserve">ANNUALISED SPREAD</t>
   </si>
   <si>
-    <t xml:space="preserve">US 3-month T-bill, 23-Oct-2026</t>
+    <t xml:space="preserve">US 3-month T-bill, 28-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Excess over T-bills (points)</t>
@@ -1074,10 +1074,10 @@
     <t xml:space="preserve">Unaffected close ($)</t>
   </si>
   <si>
-    <t xml:space="preserve">S&amp;P 500 change, 9-Apr to 23-Oct-2026</t>
-  </si>
-  <si>
-    <t xml:space="preserve">&lt;- S&amp;P 500 on 23-Oct and 9-Apr-2026</t>
+    <t xml:space="preserve">S&amp;P 500 change, 9-Apr to 28-Oct-2026</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&lt;- S&amp;P 500 on 28-Oct and 9-Apr-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Break price if the deal fails, desk assumption: unaffected moved with the S&amp;P 500 ($)</t>
@@ -1119,7 +1119,7 @@
     <t xml:space="preserve">26-Apr-2027 — extended outside date</t>
   </si>
   <si>
-    <t xml:space="preserve">On our break-price assumption the market prices about a 98% chance of completion. The spread only beats T-bills comfortably if the deal closes by the January outside date; at an April close it earns about what cash does. About 2% to gain against roughly 44% to lose if regulators or financing fail.</t>
+    <t xml:space="preserve">On our break-price assumption the market prices about a 98% chance of completion. The spread only beats T-bills comfortably if the deal closes by the January outside date; at an April close it earns about what cash does. About 2% to gain against roughly 43% to lose if regulators or financing fail.</t>
   </si>
   <si>
     <t xml:space="preserve">What it is worth, the market's verdict, and ours</t>
@@ -1266,7 +1266,7 @@
     <t xml:space="preserve">Nifty 50, 27-Apr-2026</t>
   </si>
   <si>
-    <t xml:space="preserve">Nifty 50, 23-Oct-2026</t>
+    <t xml:space="preserve">Nifty 50, 28-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">OGN unaffected market cap ($m)</t>
@@ -1281,7 +1281,7 @@
     <t xml:space="preserve">Sun relative to Nifty, 9→27 Apr (whole window from the unaffected date)</t>
   </si>
   <si>
-    <t xml:space="preserve">Sun since announcement, 27-Apr to 23-Oct-2026</t>
+    <t xml:space="preserve">Sun since announcement, 27-Apr to 28-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Nifty 50 since announcement</t>
@@ -1359,7 +1359,7 @@
     <t xml:space="preserve">Break price ↓ / OGN price →</t>
   </si>
   <si>
-    <t xml:space="preserve">Check: base break price at the 23-Oct price vs Spread &amp; Odds (must be 0)</t>
+    <t xml:space="preserve">Check: base break price at the latest price vs Spread &amp; Odds (must be 0)</t>
   </si>
   <si>
     <t xml:space="preserve">Evidence — sources for every input</t>
@@ -1446,6 +1446,18 @@
     <t xml:space="preserve">31-Jul-2026</t>
   </si>
   <si>
+    <t xml:space="preserve">ACCC review (Australia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MN-35035; notified 22-Oct-2026; Phase 1 ends 3-Dec-2026; ganirelix licensed to Ferring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ACCC acquisitions register</t>
+  </si>
+  <si>
+    <t xml:space="preserve">28-Oct-2026</t>
+  </si>
+  <si>
     <t xml:space="preserve">Seller's preliminary cost-synergy estimate</t>
   </si>
   <si>
@@ -1494,13 +1506,10 @@
     <t xml:space="preserve">Share prices, indices, FX, T-bill</t>
   </si>
   <si>
-    <t xml:space="preserve">OGN $13.75; SUN Rs 1,748; INR 94.93; 3m T-bill 4.03%; S&amp;P 500 7,623.68</t>
+    <t xml:space="preserve">OGN $13.78; SUN Rs 1,757.50; INR 95.18; 3m T-bill 4.00%; S&amp;P 500 7,743.98; Nifty 22,698.85</t>
   </si>
   <si>
     <t xml:space="preserve">NYSE / NSE closes; US Treasury 13-week yield</t>
-  </si>
-  <si>
-    <t xml:space="preserve">23-Oct-2026</t>
   </si>
   <si>
     <t xml:space="preserve">Desk assumptions</t>
@@ -1694,7 +1703,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="55">
+  <cellXfs count="56">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1904,6 +1913,10 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2311,7 +2324,7 @@
       </c>
       <c r="B17" s="9" t="n">
         <f aca="false">'Accretion-Dilution'!B32</f>
-        <v>0.115455671570174</v>
+        <v>0.115759726325178</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2320,7 +2333,7 @@
       </c>
       <c r="B18" s="10" t="n">
         <f aca="false">'Pro Forma'!B19</f>
-        <v>2.46290576518539</v>
+        <v>2.4676356440886</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2329,7 +2342,7 @@
       </c>
       <c r="B19" s="9" t="n">
         <f aca="false">'Spread &amp; Odds'!B12</f>
-        <v>0.0775757044142285</v>
+        <v>0.0725357670871125</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2338,7 +2351,7 @@
       </c>
       <c r="B20" s="9" t="n">
         <f aca="false">'Spread &amp; Odds'!B18</f>
-        <v>0.980050097070413</v>
+        <v>0.983127617193522</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3016,7 +3029,7 @@
         <v>411</v>
       </c>
       <c r="B51" s="26" t="n">
-        <v>22600</v>
+        <v>22698.85</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3061,7 +3074,7 @@
       </c>
       <c r="B56" s="9" t="n">
         <f aca="false">'Acquirer Standalone'!B5/B47-1</f>
-        <v>0.0083645803288146</v>
+        <v>0.0138448226132102</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3070,7 +3083,7 @@
       </c>
       <c r="B57" s="23" t="n">
         <f aca="false">B51/B50-1</f>
-        <v>-0.06195652625069</v>
+        <v>-0.0578536237117469</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3079,7 +3092,7 @@
       </c>
       <c r="B58" s="23" t="n">
         <f aca="false">B56-B57</f>
-        <v>0.0703211065795046</v>
+        <v>0.071698446324957</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3708,23 +3721,23 @@
       </c>
       <c r="B35" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A35*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*B$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.124251363184889</v>
+        <v>0.124578581564708</v>
       </c>
       <c r="C35" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A35*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*C$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0971051425759358</v>
+        <v>0.0973608708561842</v>
       </c>
       <c r="D35" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A35*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*D$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0699589219669825</v>
+        <v>0.0701431601476604</v>
       </c>
       <c r="E35" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A35*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*E$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0428127013580293</v>
+        <v>0.0429254494391365</v>
       </c>
       <c r="F35" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A35*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*F$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>-0.0114797398598771</v>
+        <v>-0.0115099719779112</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3733,23 +3746,23 @@
       </c>
       <c r="B36" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A36*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*B$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.146999737986485</v>
+        <v>0.147386864653467</v>
       </c>
       <c r="C36" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A36*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*C$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.119853517377531</v>
+        <v>0.120169153944943</v>
       </c>
       <c r="D36" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A36*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*D$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0927072967685781</v>
+        <v>0.0929514432364191</v>
       </c>
       <c r="E36" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A36*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*E$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0655610761596249</v>
+        <v>0.0657337325278953</v>
       </c>
       <c r="F36" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A36*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*F$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0112686349417185</v>
+        <v>0.0112983111108476</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3758,23 +3771,23 @@
       </c>
       <c r="B37" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A37*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*B$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.16974811278808</v>
+        <v>0.170195147742226</v>
       </c>
       <c r="C37" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A37*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*C$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.142601892179127</v>
+        <v>0.142977437033702</v>
       </c>
       <c r="D37" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A37*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*D$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.115455671570174</v>
+        <v>0.115759726325178</v>
       </c>
       <c r="E37" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A37*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*E$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0883094509612206</v>
+        <v>0.0885420156166541</v>
       </c>
       <c r="F37" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A37*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*F$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0340170097433141</v>
+        <v>0.0341065941996064</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3783,23 +3796,23 @@
       </c>
       <c r="B38" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A38*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*B$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.181122300188878</v>
+        <v>0.181599289286605</v>
       </c>
       <c r="C38" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A38*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*C$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.153976079579925</v>
+        <v>0.154381578578081</v>
       </c>
       <c r="D38" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A38*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*D$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.126829858970972</v>
+        <v>0.127163867869557</v>
       </c>
       <c r="E38" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A38*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*E$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0996836383620184</v>
+        <v>0.0999461571610335</v>
       </c>
       <c r="F38" s="9" t="n">
         <f aca="false">(('Accretion-Dilution'!$B$20+Synergies!$B$10*$A38*Synergies!$C$19+'Accretion-Dilution'!$B$22+'Accretion-Dilution'!$B$23-'Accretion-Dilution'!$B$10*F$34+'Accretion-Dilution'!$B$25+'Accretion-Dilution'!$B$26)*(1-'Accretion-Dilution'!$B$14)*'Accretion-Dilution'!$B$17/10/'Acquirer Standalone'!$B$6)/'Accretion-Dilution'!$B$30</f>
-        <v>0.0453911971441119</v>
+        <v>0.0455107357439858</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3834,11 +3847,12 @@
       <c r="C42" s="52" t="n">
         <v>13.5</v>
       </c>
-      <c r="D42" s="52" t="n">
-        <v>13.75</v>
+      <c r="D42" s="53" t="n">
+        <f aca="false">'Spread &amp; Odds'!B5</f>
+        <v>13.78</v>
       </c>
       <c r="E42" s="52" t="n">
-        <v>13.9</v>
+        <v>13.95</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3848,19 +3862,19 @@
       </c>
       <c r="B43" s="9" t="n">
         <f aca="false">(B$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A43)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A43)</f>
-        <v>0.911258617035624</v>
+        <v>0.910059293297112</v>
       </c>
       <c r="C43" s="9" t="n">
         <f aca="false">(C$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A43)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A43)</f>
-        <v>0.946789357069919</v>
+        <v>0.945567404581623</v>
       </c>
       <c r="D43" s="9" t="n">
         <f aca="false">(D$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A43)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A43)</f>
-        <v>0.982320097104213</v>
+        <v>0.985336489220276</v>
       </c>
       <c r="E43" s="9" t="n">
         <f aca="false">(E$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A43)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A43)</f>
-        <v>1.00363854112479</v>
+        <v>1.00948200489374</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3869,41 +3883,41 @@
       </c>
       <c r="B44" s="9" t="n">
         <f aca="false">(B$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A44)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A44)</f>
-        <v>0.910120906997619</v>
+        <v>0.908906207313742</v>
       </c>
       <c r="C44" s="9" t="n">
         <f aca="false">(C$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A44)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A44)</f>
-        <v>0.946107169340046</v>
+        <v>0.944869550794208</v>
       </c>
       <c r="D44" s="9" t="n">
         <f aca="false">(D$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A44)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A44)</f>
-        <v>0.982093431682473</v>
+        <v>0.985148495492331</v>
       </c>
       <c r="E44" s="9" t="n">
         <f aca="false">(E$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A44)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A44)</f>
-        <v>1.00368518908793</v>
+        <v>1.00960356905905</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="n">
         <f aca="false">'Spread &amp; Odds'!B17</f>
-        <v>7.71901146723793</v>
+        <v>7.84081577690317</v>
       </c>
       <c r="B45" s="9" t="n">
         <f aca="false">(B$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A45)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A45)</f>
-        <v>0.899864722877042</v>
+        <v>0.896510865905686</v>
       </c>
       <c r="C45" s="9" t="n">
         <f aca="false">(C$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A45)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A45)</f>
-        <v>0.939957409973728</v>
+        <v>0.937367824060326</v>
       </c>
       <c r="D45" s="9" t="n">
         <f aca="false">(D$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A45)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A45)</f>
-        <v>0.980050097070413</v>
+        <v>0.983127617193522</v>
       </c>
       <c r="E45" s="9" t="n">
         <f aca="false">(E$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A45)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A45)</f>
-        <v>1.00410570932843</v>
+        <v>1.01091034873868</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3912,19 +3926,19 @@
       </c>
       <c r="B46" s="9" t="n">
         <f aca="false">(B$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A46)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A46)</f>
-        <v>0.885697240420885</v>
+        <v>0.884152459301171</v>
       </c>
       <c r="C46" s="9" t="n">
         <f aca="false">(C$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A46)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A46)</f>
-        <v>0.931462378399841</v>
+        <v>0.929888450466548</v>
       </c>
       <c r="D46" s="9" t="n">
         <f aca="false">(D$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A46)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A46)</f>
-        <v>0.977227516378797</v>
+        <v>0.981112760571769</v>
       </c>
       <c r="E46" s="9" t="n">
         <f aca="false">(E$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A46)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A46)</f>
-        <v>1.00468659916617</v>
+        <v>1.01221323456422</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3933,19 +3947,19 @@
       </c>
       <c r="B47" s="9" t="n">
         <f aca="false">(B$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A47)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A47)</f>
-        <v>0.860409019275063</v>
+        <v>0.858522472420899</v>
       </c>
       <c r="C47" s="9" t="n">
         <f aca="false">(C$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A47)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A47)</f>
-        <v>0.916299187780337</v>
+        <v>0.914377045702509</v>
       </c>
       <c r="D47" s="9" t="n">
         <f aca="false">(D$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A47)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A47)</f>
-        <v>0.97218935628561</v>
+        <v>0.976934167777912</v>
       </c>
       <c r="E47" s="9" t="n">
         <f aca="false">(E$42*(1+'Spread &amp; Odds'!$B$13*'Spread &amp; Odds'!$B$11/365)-$A47)/('Spread &amp; Odds'!$B$4+'Spread &amp; Odds'!$B$6-$A47)</f>
-        <v>1.00572345738877</v>
+        <v>1.01491527760941</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3973,7 +3987,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
@@ -4015,251 +4029,270 @@
       </c>
     </row>
     <row r="5" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="53" t="s">
+      <c r="A5" s="54" t="s">
         <v>448</v>
       </c>
-      <c r="B5" s="53" t="s">
+      <c r="B5" s="54" t="s">
         <v>449</v>
       </c>
-      <c r="C5" s="53" t="s">
+      <c r="C5" s="54" t="s">
         <v>450</v>
       </c>
-      <c r="D5" s="53" t="s">
+      <c r="D5" s="54" t="s">
         <v>451</v>
       </c>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
-      <c r="G5" s="54"/>
-      <c r="H5" s="54"/>
-      <c r="I5" s="54"/>
+      <c r="E5" s="55"/>
+      <c r="F5" s="55"/>
+      <c r="G5" s="55"/>
+      <c r="H5" s="55"/>
+      <c r="I5" s="55"/>
     </row>
     <row r="6" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="53" t="s">
+      <c r="A6" s="54" t="s">
         <v>452</v>
       </c>
-      <c r="B6" s="53" t="s">
+      <c r="B6" s="54" t="s">
         <v>453</v>
       </c>
-      <c r="C6" s="53" t="s">
+      <c r="C6" s="54" t="s">
         <v>454</v>
       </c>
-      <c r="D6" s="53" t="s">
+      <c r="D6" s="54" t="s">
         <v>451</v>
       </c>
-      <c r="E6" s="54"/>
-      <c r="F6" s="54"/>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
-      <c r="I6" s="54"/>
+      <c r="E6" s="55"/>
+      <c r="F6" s="55"/>
+      <c r="G6" s="55"/>
+      <c r="H6" s="55"/>
+      <c r="I6" s="55"/>
     </row>
     <row r="7" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="53" t="s">
+      <c r="A7" s="54" t="s">
         <v>455</v>
       </c>
-      <c r="B7" s="53" t="s">
+      <c r="B7" s="54" t="s">
         <v>456</v>
       </c>
-      <c r="C7" s="53" t="s">
+      <c r="C7" s="54" t="s">
         <v>457</v>
       </c>
-      <c r="D7" s="53" t="s">
+      <c r="D7" s="54" t="s">
         <v>451</v>
       </c>
-      <c r="E7" s="54"/>
-      <c r="F7" s="54"/>
-      <c r="G7" s="54"/>
-      <c r="H7" s="54"/>
-      <c r="I7" s="54"/>
+      <c r="E7" s="55"/>
+      <c r="F7" s="55"/>
+      <c r="G7" s="55"/>
+      <c r="H7" s="55"/>
+      <c r="I7" s="55"/>
     </row>
     <row r="8" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="53" t="s">
+      <c r="A8" s="54" t="s">
         <v>458</v>
       </c>
-      <c r="B8" s="53" t="s">
+      <c r="B8" s="54" t="s">
         <v>459</v>
       </c>
-      <c r="C8" s="53" t="s">
+      <c r="C8" s="54" t="s">
         <v>460</v>
       </c>
-      <c r="D8" s="53" t="s">
+      <c r="D8" s="54" t="s">
         <v>451</v>
       </c>
-      <c r="E8" s="54"/>
-      <c r="F8" s="54"/>
-      <c r="G8" s="54"/>
-      <c r="H8" s="54"/>
-      <c r="I8" s="54"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
     </row>
     <row r="9" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="53" t="s">
+      <c r="A9" s="54" t="s">
         <v>461</v>
       </c>
-      <c r="B9" s="53" t="s">
+      <c r="B9" s="54" t="s">
         <v>462</v>
       </c>
-      <c r="C9" s="53" t="s">
+      <c r="C9" s="54" t="s">
         <v>463</v>
       </c>
-      <c r="D9" s="53" t="s">
+      <c r="D9" s="54" t="s">
         <v>451</v>
       </c>
-      <c r="E9" s="54"/>
-      <c r="F9" s="54"/>
-      <c r="G9" s="54"/>
-      <c r="H9" s="54"/>
-      <c r="I9" s="54"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
+      <c r="H9" s="55"/>
+      <c r="I9" s="55"/>
     </row>
     <row r="10" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="53" t="s">
+      <c r="A10" s="54" t="s">
         <v>464</v>
       </c>
-      <c r="B10" s="53" t="s">
+      <c r="B10" s="54" t="s">
         <v>462</v>
       </c>
-      <c r="C10" s="53" t="s">
+      <c r="C10" s="54" t="s">
         <v>465</v>
       </c>
-      <c r="D10" s="53" t="s">
+      <c r="D10" s="54" t="s">
         <v>466</v>
       </c>
-      <c r="E10" s="54"/>
-      <c r="F10" s="54"/>
-      <c r="G10" s="54"/>
-      <c r="H10" s="54"/>
-      <c r="I10" s="54"/>
+      <c r="E10" s="55"/>
+      <c r="F10" s="55"/>
+      <c r="G10" s="55"/>
+      <c r="H10" s="55"/>
+      <c r="I10" s="55"/>
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="54" t="s">
         <v>467</v>
       </c>
-      <c r="B11" s="53" t="s">
+      <c r="B11" s="54" t="s">
         <v>468</v>
       </c>
-      <c r="C11" s="53" t="s">
+      <c r="C11" s="54" t="s">
         <v>469</v>
       </c>
-      <c r="D11" s="53" t="s">
+      <c r="D11" s="54" t="s">
         <v>470</v>
       </c>
-      <c r="E11" s="54"/>
-      <c r="F11" s="54"/>
-      <c r="G11" s="54"/>
-      <c r="H11" s="54"/>
-      <c r="I11" s="54"/>
-    </row>
-    <row r="12" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="53" t="s">
+      <c r="E11" s="55"/>
+      <c r="F11" s="55"/>
+      <c r="G11" s="55"/>
+      <c r="H11" s="55"/>
+      <c r="I11" s="55"/>
+    </row>
+    <row r="12" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="54" t="s">
         <v>471</v>
       </c>
-      <c r="B12" s="53" t="s">
+      <c r="B12" s="54" t="s">
         <v>472</v>
       </c>
-      <c r="C12" s="53" t="s">
+      <c r="C12" s="54" t="s">
         <v>473</v>
       </c>
-      <c r="D12" s="53" t="s">
+      <c r="D12" s="54" t="s">
         <v>474</v>
       </c>
-      <c r="E12" s="54"/>
-      <c r="F12" s="54"/>
-      <c r="G12" s="54"/>
-      <c r="H12" s="54"/>
-      <c r="I12" s="54"/>
-    </row>
-    <row r="13" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="53" t="s">
+      <c r="E12" s="55"/>
+      <c r="F12" s="55"/>
+      <c r="G12" s="55"/>
+      <c r="H12" s="55"/>
+      <c r="I12" s="55"/>
+    </row>
+    <row r="13" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="54" t="s">
         <v>475</v>
       </c>
-      <c r="B13" s="53" t="s">
+      <c r="B13" s="54" t="s">
         <v>476</v>
       </c>
-      <c r="C13" s="53" t="s">
+      <c r="C13" s="54" t="s">
         <v>477</v>
       </c>
-      <c r="D13" s="53" t="s">
+      <c r="D13" s="54" t="s">
         <v>478</v>
       </c>
-      <c r="E13" s="54"/>
-      <c r="F13" s="54"/>
-      <c r="G13" s="54"/>
-      <c r="H13" s="54"/>
-      <c r="I13" s="54"/>
-    </row>
-    <row r="14" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="53" t="s">
+      <c r="E13" s="55"/>
+      <c r="F13" s="55"/>
+      <c r="G13" s="55"/>
+      <c r="H13" s="55"/>
+      <c r="I13" s="55"/>
+    </row>
+    <row r="14" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="54" t="s">
         <v>479</v>
       </c>
-      <c r="B14" s="53" t="s">
-        <v>476</v>
-      </c>
-      <c r="C14" s="53" t="s">
+      <c r="B14" s="54" t="s">
         <v>480</v>
       </c>
-      <c r="D14" s="53" t="s">
+      <c r="C14" s="54" t="s">
         <v>481</v>
       </c>
-      <c r="E14" s="54"/>
-      <c r="F14" s="54"/>
-      <c r="G14" s="54"/>
-      <c r="H14" s="54"/>
-      <c r="I14" s="54"/>
+      <c r="D14" s="54" t="s">
+        <v>482</v>
+      </c>
+      <c r="E14" s="55"/>
+      <c r="F14" s="55"/>
+      <c r="G14" s="55"/>
+      <c r="H14" s="55"/>
+      <c r="I14" s="55"/>
     </row>
     <row r="15" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="53" t="s">
-        <v>482</v>
-      </c>
-      <c r="B15" s="53" t="s">
+      <c r="A15" s="54" t="s">
         <v>483</v>
       </c>
-      <c r="C15" s="53" t="s">
+      <c r="B15" s="54" t="s">
+        <v>480</v>
+      </c>
+      <c r="C15" s="54" t="s">
         <v>484</v>
       </c>
-      <c r="D15" s="53" t="s">
+      <c r="D15" s="54" t="s">
         <v>485</v>
       </c>
-      <c r="E15" s="54"/>
-      <c r="F15" s="54"/>
-      <c r="G15" s="54"/>
-      <c r="H15" s="54"/>
-      <c r="I15" s="54"/>
-    </row>
-    <row r="16" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="53" t="s">
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="55"/>
+      <c r="H15" s="55"/>
+      <c r="I15" s="55"/>
+    </row>
+    <row r="16" customFormat="false" ht="12.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="54" t="s">
         <v>486</v>
       </c>
-      <c r="B16" s="53" t="s">
+      <c r="B16" s="54" t="s">
         <v>487</v>
       </c>
-      <c r="C16" s="53" t="s">
+      <c r="C16" s="54" t="s">
         <v>488</v>
       </c>
-      <c r="D16" s="53" t="s">
+      <c r="D16" s="54" t="s">
         <v>489</v>
       </c>
-      <c r="E16" s="54"/>
-      <c r="F16" s="54"/>
-      <c r="G16" s="54"/>
-      <c r="H16" s="54"/>
-      <c r="I16" s="54"/>
-    </row>
-    <row r="17" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="53" t="s">
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="55"/>
+      <c r="H16" s="55"/>
+      <c r="I16" s="55"/>
+    </row>
+    <row r="17" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="54" t="s">
         <v>490</v>
       </c>
-      <c r="B17" s="53" t="s">
+      <c r="B17" s="54" t="s">
         <v>491</v>
       </c>
-      <c r="C17" s="53" t="s">
+      <c r="C17" s="54" t="s">
         <v>492</v>
       </c>
-      <c r="D17" s="53" t="s">
+      <c r="D17" s="54" t="s">
+        <v>474</v>
+      </c>
+      <c r="E17" s="55"/>
+      <c r="F17" s="55"/>
+      <c r="G17" s="55"/>
+      <c r="H17" s="55"/>
+      <c r="I17" s="55"/>
+    </row>
+    <row r="18" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="54" t="s">
         <v>493</v>
       </c>
-      <c r="E17" s="54"/>
-      <c r="F17" s="54"/>
-      <c r="G17" s="54"/>
-      <c r="H17" s="54"/>
-      <c r="I17" s="54"/>
+      <c r="B18" s="54" t="s">
+        <v>494</v>
+      </c>
+      <c r="C18" s="54" t="s">
+        <v>495</v>
+      </c>
+      <c r="D18" s="54" t="s">
+        <v>496</v>
+      </c>
+      <c r="E18" s="55"/>
+      <c r="F18" s="55"/>
+      <c r="G18" s="55"/>
+      <c r="H18" s="55"/>
+      <c r="I18" s="55"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -4415,7 +4448,7 @@
       <c r="G11" s="12"/>
       <c r="H11" s="12"/>
     </row>
-    <row r="12" customFormat="false" ht="39" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" customFormat="false" ht="51.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="6" t="s">
         <v>55</v>
       </c>
@@ -5590,7 +5623,7 @@
         <v>170</v>
       </c>
       <c r="B5" s="26" t="n">
-        <v>1748</v>
+        <v>1757.5</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5607,7 +5640,7 @@
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">B5*B6</f>
-        <v>419397.64</v>
+        <v>421676.975</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5696,7 +5729,7 @@
       </c>
       <c r="B18" s="27" t="n">
         <f aca="false">B5/B8</f>
-        <v>36.5384615384615</v>
+        <v>36.7370401337793</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5704,7 +5737,7 @@
         <v>184</v>
       </c>
       <c r="B19" s="26" t="n">
-        <v>94.93</v>
+        <v>95.18</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5730,7 +5763,7 @@
       </c>
       <c r="B23" s="8" t="n">
         <f aca="false">Synergies!B6*B19/10</f>
-        <v>111542.75</v>
+        <v>111836.5</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5739,7 +5772,7 @@
       </c>
       <c r="B24" s="19" t="n">
         <f aca="false">B23-B22</f>
-        <v>789.012499999997</v>
+        <v>1082.7625</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6762,7 +6795,7 @@
       </c>
       <c r="B17" s="36" t="n">
         <f aca="false">'Acquirer Standalone'!B19</f>
-        <v>94.93</v>
+        <v>95.18</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6936,15 +6969,15 @@
       </c>
       <c r="B29" s="36" t="n">
         <f aca="false">B28*$B$17/10/'Acquirer Standalone'!$B$6</f>
-        <v>6.58905517650982</v>
+        <v>6.6064075813779</v>
       </c>
       <c r="C29" s="36" t="n">
         <f aca="false">C28*$B$17/10/'Acquirer Standalone'!$B$6</f>
-        <v>12.6277711561706</v>
+        <v>12.6610266369358</v>
       </c>
       <c r="D29" s="36" t="n">
         <f aca="false">D28*$B$17/10/'Acquirer Standalone'!$B$6</f>
-        <v>23.4885576355604</v>
+        <v>23.5504152086025</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6970,15 +7003,15 @@
       </c>
       <c r="B31" s="37" t="n">
         <f aca="false">B30+B29</f>
-        <v>63.6590551765098</v>
+        <v>63.6764075813779</v>
       </c>
       <c r="C31" s="37" t="n">
         <f aca="false">C30+C29</f>
-        <v>74.1577711561706</v>
+        <v>74.1910266369358</v>
       </c>
       <c r="D31" s="37" t="n">
         <f aca="false">D30+D29</f>
-        <v>89.5285576355604</v>
+        <v>89.5904152086025</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6987,15 +7020,15 @@
       </c>
       <c r="B32" s="28" t="n">
         <f aca="false">B31/B30-1</f>
-        <v>0.115455671570174</v>
+        <v>0.115759726325178</v>
       </c>
       <c r="C32" s="28" t="n">
         <f aca="false">C31/C30-1</f>
-        <v>0.205229500344069</v>
+        <v>0.205769976221937</v>
       </c>
       <c r="D32" s="28" t="n">
         <f aca="false">D31/D30-1</f>
-        <v>0.355671678309515</v>
+        <v>0.356608346586955</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7004,15 +7037,15 @@
       </c>
       <c r="B33" s="9" t="n">
         <f aca="false">(B30+(B27-B22-B26)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/B30-1</f>
-        <v>0.466430597080506</v>
+        <v>0.467658951123171</v>
       </c>
       <c r="C33" s="9" t="n">
         <f aca="false">(C30+(C27-C22-C26)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/C30-1</f>
-        <v>0.530764020072245</v>
+        <v>0.532161797434702</v>
       </c>
       <c r="D33" s="9" t="n">
         <f aca="false">(D30+(D27-D22-D26)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/D30-1</f>
-        <v>0.580340666788716</v>
+        <v>0.581869005213842</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7021,15 +7054,15 @@
       </c>
       <c r="B34" s="9" t="n">
         <f aca="false">(B30+(B27-B21-B22)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/B30-1</f>
-        <v>0.160952421173365</v>
+        <v>0.161376292502696</v>
       </c>
       <c r="C34" s="9" t="n">
         <f aca="false">(C30+(C27-C21-C22)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/C30-1</f>
-        <v>0.18834993265446</v>
+        <v>0.188845955862756</v>
       </c>
       <c r="D34" s="9" t="n">
         <f aca="false">(D30+(D27-D21-D22)*(1-$B$14)*$B$17/10/'Acquirer Standalone'!$B$6)/D30-1</f>
-        <v>0.198403386374074</v>
+        <v>0.198925885548134</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7051,7 +7084,7 @@
       </c>
       <c r="B37" s="23" t="n">
         <f aca="false">B33</f>
-        <v>0.466430597080506</v>
+        <v>0.467658951123171</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7060,7 +7093,7 @@
       </c>
       <c r="B38" s="9" t="n">
         <f aca="false">(B30+(B27-B22-B26-B21*(1-C38))*(1-B14)*B17/10/'Acquirer Standalone'!B6)/B30-1</f>
-        <v>0.443682222278911</v>
+        <v>0.444850668034412</v>
       </c>
       <c r="C38" s="24" t="n">
         <v>0.5</v>
@@ -7326,7 +7359,7 @@
       </c>
       <c r="B13" s="8" t="n">
         <f aca="false">'Acquirer Standalone'!B13*10/'Acquirer Standalone'!B19</f>
-        <v>487.411777098915</v>
+        <v>486.131540239546</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7335,7 +7368,7 @@
       </c>
       <c r="B14" s="8" t="n">
         <f aca="false">-('Acquirer Standalone'!B12*10/'Acquirer Standalone'!B19-B5)</f>
-        <v>-354.340040029495</v>
+        <v>-347.499474679554</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7353,7 +7386,7 @@
       </c>
       <c r="B16" s="16" t="n">
         <f aca="false">SUM(B12:B15)</f>
-        <v>9442.67173706942</v>
+        <v>9448.23206555999</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7362,7 +7395,7 @@
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">'Acquirer Standalone'!B14*10/'Acquirer Standalone'!B19</f>
-        <v>1939.95575687349</v>
+        <v>1934.8602647615</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7380,7 +7413,7 @@
       </c>
       <c r="B19" s="38" t="n">
         <f aca="false">B16/(B17+B18)</f>
-        <v>2.46290576518539</v>
+        <v>2.4676356440886</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7397,7 +7430,7 @@
       </c>
       <c r="B21" s="23" t="n">
         <f aca="false">B18/(B17+B18)</f>
-        <v>0.49400674397571</v>
+        <v>0.494664173940016</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7460,7 +7493,7 @@
         <v>336</v>
       </c>
       <c r="B5" s="13" t="n">
-        <v>13.75</v>
+        <v>13.78</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7477,7 +7510,7 @@
       </c>
       <c r="B7" s="39" t="n">
         <f aca="false">B4+B6-B5</f>
-        <v>0.27</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7486,7 +7519,7 @@
       </c>
       <c r="B8" s="18" t="n">
         <f aca="false">B7/B5</f>
-        <v>0.0196363636363636</v>
+        <v>0.0174165457184325</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7494,7 +7527,7 @@
         <v>340</v>
       </c>
       <c r="B9" s="40" t="n">
-        <v>46318</v>
+        <v>46323</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7511,7 +7544,7 @@
       </c>
       <c r="B11" s="41" t="n">
         <f aca="false">B10-B9</f>
-        <v>95</v>
+        <v>90</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7520,7 +7553,7 @@
       </c>
       <c r="B12" s="28" t="n">
         <f aca="false">(1+B8)^(365/B11)-1</f>
-        <v>0.0775757044142285</v>
+        <v>0.0725357670871125</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7528,7 +7561,7 @@
         <v>344</v>
       </c>
       <c r="B13" s="42" t="n">
-        <v>0.04032</v>
+        <v>0.03995</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7537,7 +7570,7 @@
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">B12-B13</f>
-        <v>0.0372557044142285</v>
+        <v>0.0325857670871125</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7555,10 +7588,10 @@
       </c>
       <c r="B16" s="23" t="n">
         <f aca="false">C16/D16-1</f>
-        <v>0.117078359947602</v>
+        <v>0.134705611708129</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>7623.68</v>
+        <v>7743.98</v>
       </c>
       <c r="D16" s="26" t="n">
         <v>6824.66</v>
@@ -7573,7 +7606,7 @@
       </c>
       <c r="B17" s="39" t="n">
         <f aca="false">B15*(1+B16)</f>
-        <v>7.71901146723793</v>
+        <v>7.84081577690317</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7582,7 +7615,7 @@
       </c>
       <c r="B18" s="23" t="n">
         <f aca="false">(B5*(1+B13*B11/365)-B17)/(B4+B6-B17)</f>
-        <v>0.980050097070413</v>
+        <v>0.983127617193522</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7591,7 +7624,7 @@
       </c>
       <c r="B19" s="23" t="n">
         <f aca="false">B17/B5-1</f>
-        <v>-0.438617347837242</v>
+        <v>-0.431000306465662</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7600,7 +7633,7 @@
       </c>
       <c r="B20" s="18" t="n">
         <f aca="false">B8</f>
-        <v>0.0196363636363636</v>
+        <v>0.0174165457184325</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7609,7 +7642,7 @@
       </c>
       <c r="B21" s="43" t="n">
         <f aca="false">-B19/B20</f>
-        <v>22.3369945657855</v>
+        <v>24.7466009295701</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -7645,15 +7678,15 @@
       </c>
       <c r="B25" s="41" t="n">
         <f aca="false">E25-$B$9</f>
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C25" s="23" t="n">
         <f aca="false">(1+$B$8)^(365/B25)-1</f>
-        <v>0.0775757044142285</v>
+        <v>0.0725357670871125</v>
       </c>
       <c r="D25" s="44" t="n">
         <f aca="false">C25-$B$13</f>
-        <v>0.0372557044142285</v>
+        <v>0.0325857670871125</v>
       </c>
       <c r="E25" s="40" t="n">
         <v>46413</v>
@@ -7665,15 +7698,15 @@
       </c>
       <c r="B26" s="41" t="n">
         <f aca="false">E26-$B$9</f>
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="C26" s="23" t="n">
         <f aca="false">(1+$B$8)^(365/B26)-1</f>
-        <v>0.0456516929543462</v>
+        <v>0.0417730552940061</v>
       </c>
       <c r="D26" s="44" t="n">
         <f aca="false">C26-$B$13</f>
-        <v>0.00533169295434623</v>
+        <v>0.0018230552940061</v>
       </c>
       <c r="E26" s="40" t="n">
         <v>46477</v>
@@ -7685,15 +7718,15 @@
       </c>
       <c r="B27" s="41" t="n">
         <f aca="false">E27-$B$9</f>
-        <v>185</v>
+        <v>180</v>
       </c>
       <c r="C27" s="23" t="n">
         <f aca="false">(1+$B$8)^(365/B27)-1</f>
-        <v>0.0391120453064238</v>
+        <v>0.0356330272288117</v>
       </c>
       <c r="D27" s="44" t="n">
         <f aca="false">C27-$B$13</f>
-        <v>-0.00120795469357624</v>
+        <v>-0.00431697277118832</v>
       </c>
       <c r="E27" s="40" t="n">
         <v>46503</v>

</xml_diff>